<commit_message>
actualizacion de excel contacto
</commit_message>
<xml_diff>
--- a/data/contacto.xlsx
+++ b/data/contacto.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luigi\Documents\LAO\Formacion\202602 Data Storytelling\Storytelling Project\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luigi\Documents\LAO\GB Laostat\data-storytelling-workshop\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A76DEB-BE65-4E96-B0FB-CDA3271C5E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F57967E-B990-4888-B11C-AC48EA99105D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2ED19271-0958-4AA1-8C04-8B0EFDA7F98D}"/>
   </bookViews>
@@ -53,13 +53,13 @@
     <t>Departemento Papeleria</t>
   </si>
   <si>
-    <t>Departamento de Mobilidario</t>
-  </si>
-  <si>
     <t>Logística</t>
   </si>
   <si>
     <t>area</t>
+  </si>
+  <si>
+    <t>Departamento de Mobiliario</t>
   </si>
 </sst>
 </file>
@@ -463,7 +463,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="30.6">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -496,7 +496,7 @@
     </row>
     <row r="4" spans="1:3" ht="15.6">
       <c r="A4" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B4" s="3">
         <v>0.69</v>
@@ -507,7 +507,7 @@
     </row>
     <row r="5" spans="1:3" ht="15.6">
       <c r="A5" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5" s="3">
         <v>0.94</v>

</xml_diff>